<commit_message>
Opcion de editar en los item
</commit_message>
<xml_diff>
--- a/docs/Inventario_Insumos_2026.xlsx
+++ b/docs/Inventario_Insumos_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Carlos Orozco DTI\Documents\Control-Avales-DSST\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC6DEA7-7982-423A-8BA8-C82184708D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC3F8D54-FA47-4246-855B-99A757EE4561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mantenimiento" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -886,7 +883,7 @@
         <v>36</v>
       </c>
       <c r="I7" s="4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -898,12 +895,12 @@
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4">
-        <f t="shared" ref="S7:S20" si="0">SUM(G7:R7)</f>
-        <v>37</v>
+        <f>SUM(G7:R7)</f>
+        <v>49</v>
       </c>
       <c r="T7" s="4">
-        <f t="shared" ref="T7:T20" si="1">(E7+F7)-S7</f>
-        <v>67</v>
+        <f>(E7+F7)-S7</f>
+        <v>55</v>
       </c>
       <c r="U7" s="4">
         <v>500</v>
@@ -945,11 +942,11 @@
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="S7:S20" si="0">SUM(G8:R8)</f>
         <v>0</v>
       </c>
       <c r="T8" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="T7:T20" si="1">(E8+F8)-S8</f>
         <v>3</v>
       </c>
       <c r="U8" s="4">
@@ -1031,7 +1028,7 @@
         <v>12</v>
       </c>
       <c r="I10" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -1044,11 +1041,11 @@
       <c r="R10" s="4"/>
       <c r="S10" s="4">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T10" s="4">
         <f t="shared" si="1"/>
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="U10" s="4">
         <v>0</v>
@@ -1127,7 +1124,7 @@
         <v>8</v>
       </c>
       <c r="I12" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
@@ -1140,11 +1137,11 @@
       <c r="R12" s="4"/>
       <c r="S12" s="4">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="T12" s="4">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="U12" s="4">
         <v>36</v>
@@ -1269,7 +1266,9 @@
       <c r="H15" s="4">
         <v>1</v>
       </c>
-      <c r="I15" s="4"/>
+      <c r="I15" s="4">
+        <v>4</v>
+      </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
@@ -1281,11 +1280,11 @@
       <c r="R15" s="4"/>
       <c r="S15" s="4">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="T15" s="4">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="U15" s="4">
         <v>0</v>
@@ -1536,7 +1535,7 @@
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="145" scale="66" orientation="landscape" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="S7:S20" formulaRange="1"/>
+    <ignoredError sqref="S8:S20" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>